<commit_message>
Chi Phí Cơ Sở: số lớn trong .xlsx là dạng khoa học — bỏ chữ E làm 564.538.680đ thành 5,65đ
Đối chiếu từng dòng với hệ cũ mới thấy: không phải đọc THIẾU dòng mà đọc SAI giá trị.

  bảng tính      trong file .xlsx   app đọc ra
  564.538.680    5.6453868E8        5,65
  549.256.680    5.4925668E8        5,49
   10.800.000    1.08E7             1,09

Google xuất .xlsx ghi số lớn theo dạng khoa học. VHCP_Util::doc_so() kết thúc bằng
preg_replace('/[^0-9.\-]/','') để dọn ký tự lạ — thao tác đó bỏ luôn chữ E, nên
5.6453868E8 thành 5.64538688. Nhận dạng dạng khoa học TRƯỚC mọi xử lý dấu nghìn /
dấu thập phân (chuỗi kiểu này không bao giờ là dấu nghìn), chấp cả 5,6453868E8 kiểu
dấu phẩy thập phân và số âm.

File mẫu test thêm một dòng mang đúng giá trị 5.4925668E8 để chạy hết đường từ đọc
.xlsx tới tổng trong sổ chi phí.

663 phép thử đạt; bench không màn nào đọc lặp.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K1rxYgpiPcxzLLvMyvVXic
</commit_message>
<xml_diff>
--- a/tools/test/fixtures/nha-ma-ba-ria.xlsx
+++ b/tools/test/fixtures/nha-ma-ba-ria.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>🏗 SETUP LẮP ĐẶT: NHÀ MA BÀ RỊA</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Thi công hệ vách (trọn gói)</t>
   </si>
 </sst>
 </file>
@@ -130,13 +133,27 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" s="3" customFormat="1">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="3" t="str">
-        <v/>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>5.4925668E8</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>5.4925668E8</v>
+      </c>
+      <c r="F7">
+        <v>5.4925668E8</v>
+      </c>
+      <c r="G7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="8" s="3" customFormat="1">
@@ -490,6 +507,15 @@
         <v/>
       </c>
     </row>
+    <row r="47" s="3" customFormat="1">
+      <c r="A47" s="3"/>
+      <c r="B47" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" s="3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>